<commit_message>
2025_12 exam is over"
</commit_message>
<xml_diff>
--- a/READING/7_19_07.xlsx
+++ b/READING/7_19_07.xlsx
@@ -466,16 +466,16 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>みつける</t>
+          <t>ながめる</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>找到</t>
+          <t>眺望</t>
         </is>
       </c>
       <c r="D2" t="inlineStr"/>
@@ -483,100 +483,84 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>出来事にあう</t>
+          <t>なにもかも</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>遇到事情</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>できごとにあう</t>
-        </is>
-      </c>
+          <t>一切，所有</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>知り合った</t>
+          <t>やがて</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>结识，认识</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>しりあった</t>
-        </is>
-      </c>
+          <t>不久，马上</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>時間をとられる</t>
+          <t>たしかめる</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>被占用时间</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>じかんをとられる</t>
-        </is>
-      </c>
+          <t>确认</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>お得</t>
+          <t>なんとかなる</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>划算；优惠</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>おとく</t>
-        </is>
-      </c>
+          <t>总会有办法的</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>あとで</t>
+          <t>なんらか</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>之后，待会儿</t>
+          <t>某些，某种</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
@@ -584,16 +568,16 @@
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>ながめる</t>
+          <t>あたりまえ</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>眺望</t>
+          <t>理所当然</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
@@ -601,16 +585,16 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>やがて</t>
+          <t>〜につきまして</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>不久，马上</t>
+          <t>关于...（「について」的礼貌说法）</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
@@ -618,16 +602,16 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>N+のかをつける</t>
+          <t>やってくる</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>增强…能力</t>
+          <t>到来；做过来</t>
         </is>
       </c>
       <c r="D10" t="inlineStr"/>
@@ -635,16 +619,16 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>および</t>
+          <t>なおす</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>以及，和</t>
+          <t>修理；改正</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
@@ -652,16 +636,16 @@
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>いたす</t>
+          <t>せずに</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>“する”的自谦语</t>
+          <t>不做...就...（书面语）</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
@@ -669,16 +653,16 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>それぞれ</t>
+          <t>いたす</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>各自，分别</t>
+          <t>“する”的自谦语</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
@@ -686,58 +670,50 @@
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>〜を付けた</t>
+          <t>あらかじめ</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>附带着</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>〜をつけた</t>
-        </is>
-      </c>
+          <t>预先，事先</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>〜に限り</t>
+          <t>それなのに</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>限于...，只有...</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>〜にかぎり</t>
-        </is>
-      </c>
+          <t>尽管如此，可是...</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>どちらも…</t>
+          <t>あふれる</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>无论哪一个都…</t>
+          <t>溢出，充满</t>
         </is>
       </c>
       <c r="D16" t="inlineStr"/>
@@ -745,16 +721,16 @@
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>ずつ</t>
+          <t>のほかに</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>每...</t>
+          <t>除...之外</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
@@ -762,16 +738,16 @@
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>ぜひ</t>
+          <t>〜のせいにする</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>一定，务必</t>
+          <t>把责任归因于…</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
@@ -779,58 +755,54 @@
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>あて先</t>
+          <t>かならずしも〜ではない</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>收件人地址</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>あてさき</t>
-        </is>
-      </c>
+          <t>未必，不一定</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>数量詞+ずつ</t>
+          <t>手応え</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>每...（数量）</t>
+          <t>手感；反应，效果</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>すうりょうし+ずつ</t>
+          <t>てごたえ</t>
         </is>
       </c>
       <c r="E20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>のうち</t>
+          <t>あとで</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>...之中</t>
+          <t>之后，待会儿</t>
         </is>
       </c>
       <c r="D21" t="inlineStr"/>
@@ -838,50 +810,58 @@
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>あたりまえ</t>
+          <t>知り合った</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>理所当然</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr"/>
+          <t>结识，认识</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>しりあった</t>
+        </is>
+      </c>
       <c r="E22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>かならずしも〜ではない</t>
+          <t>着実に</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>未必，不一定</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr"/>
+          <t>切实地，踏实地</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>ちゃくじつに</t>
+        </is>
+      </c>
       <c r="E23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>なにか</t>
+          <t>Vる+のか</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>什么，某些</t>
+          <t>是否…</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
@@ -889,54 +869,58 @@
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>身につく</t>
+          <t>あて先</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>掌握，学会</t>
+          <t>收件人地址</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>みにつく</t>
+          <t>あてさき</t>
         </is>
       </c>
       <c r="E25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>ふだん</t>
+          <t>の方が</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>平时，平常</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr"/>
+          <t>更加</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>のほうが</t>
+        </is>
+      </c>
       <c r="E26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>しっかりと</t>
+          <t>つかむ</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>踏实地</t>
+          <t>抓住，掌握</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
@@ -944,54 +928,54 @@
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>とらえる</t>
+          <t>〜を付けた</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>捕捉，理解</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr"/>
+          <t>附带着</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>〜をつけた</t>
+        </is>
+      </c>
       <c r="E28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>手応え</t>
+          <t>〜ないだろうか</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>手感；反应，效果</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>てごたえ</t>
-        </is>
-      </c>
+          <t>是否…</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>〜につきまして</t>
+          <t>みつける</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>关于...（「について」的礼貌说法）</t>
+          <t>找到</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
@@ -999,37 +983,33 @@
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>一気に</t>
+          <t>ずつ</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>一口气地</t>
-        </is>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>いっきに</t>
-        </is>
-      </c>
+          <t>每...</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>たしかめる</t>
+          <t>にかかわる</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>确认</t>
+          <t>关系到...，涉及到...</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
@@ -1037,86 +1017,74 @@
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>売り行き</t>
+          <t>N+のかをつける</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>销路，销售</t>
-        </is>
-      </c>
-      <c r="D33" t="inlineStr">
-        <is>
-          <t>うりいき</t>
-        </is>
-      </c>
+          <t>增强…能力</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>追いつく</t>
+          <t>〜とする</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>追上，赶上</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>おいつく</t>
-        </is>
-      </c>
+          <t>假如…</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>納品</t>
+          <t>出来事にあう</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>交货</t>
+          <t>遇到事情</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>のうひん</t>
+          <t>できごとにあう</t>
         </is>
       </c>
       <c r="E35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>改める</t>
+          <t>しっかりと</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>重新</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>あらためる</t>
-        </is>
-      </c>
+          <t>踏实地</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr"/>
     </row>
     <row r="37">
@@ -1125,17 +1093,17 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>監督</t>
+          <t>与える</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>监督；导演</t>
+          <t>给予，赋予</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>かんとく</t>
+          <t>あたえる</t>
         </is>
       </c>
       <c r="E37" t="inlineStr"/>
@@ -1146,17 +1114,17 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>相性が悪い</t>
+          <t>監督</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>(两人)合不来</t>
+          <t>监督；导演</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>あいしょうがわるい</t>
+          <t>かんとく</t>
         </is>
       </c>
       <c r="E38" t="inlineStr"/>
@@ -1167,38 +1135,34 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>活躍</t>
+          <t>そうして〜</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>活跃，大显身手</t>
-        </is>
-      </c>
-      <c r="D39" t="inlineStr">
-        <is>
-          <t>かつやく</t>
-        </is>
-      </c>
+          <t>这么做…</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>周り</t>
+          <t>追いつく</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>周围</t>
+          <t>追上，赶上</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>まわり</t>
+          <t>おいつく</t>
         </is>
       </c>
       <c r="E40" t="inlineStr"/>
@@ -1209,15 +1173,19 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>〜のせいにする</t>
+          <t>時間をとられる</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>把责任归因于…</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr"/>
+          <t>被占用时间</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>じかんをとられる</t>
+        </is>
+      </c>
       <c r="E41" t="inlineStr"/>
     </row>
     <row r="42">
@@ -1226,15 +1194,19 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>しかも</t>
+          <t>一気に</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>而且</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr"/>
+          <t>一口气地</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>いっきに</t>
+        </is>
+      </c>
       <c r="E42" t="inlineStr"/>
     </row>
     <row r="43">
@@ -1243,15 +1215,19 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>ととらえる</t>
+          <t>納品</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>视为...，理解为...</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr"/>
+          <t>交货</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>のうひん</t>
+        </is>
+      </c>
       <c r="E43" t="inlineStr"/>
     </row>
     <row r="44">
@@ -1260,19 +1236,15 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>の方が</t>
+          <t>ふだん</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>更加</t>
-        </is>
-      </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>のほうが</t>
-        </is>
-      </c>
+          <t>平时，平常</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr"/>
       <c r="E44" t="inlineStr"/>
     </row>
     <row r="45">
@@ -1281,17 +1253,17 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>受け取る</t>
+          <t>売り行き</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>接收，领取；理解</t>
+          <t>销路，销售</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>うけとる</t>
+          <t>うりいき</t>
         </is>
       </c>
       <c r="E45" t="inlineStr"/>
@@ -1302,29 +1274,33 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>にかかわる</t>
+          <t>お得</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>关系到...，涉及到...</t>
-        </is>
-      </c>
-      <c r="D46" t="inlineStr"/>
+          <t>划算；优惠</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>おとく</t>
+        </is>
+      </c>
       <c r="E46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>によって</t>
+          <t>いずれ</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>根据...；由于...</t>
+          <t>反正，早晚</t>
         </is>
       </c>
       <c r="D47" t="inlineStr"/>
@@ -1336,12 +1312,12 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>とよい</t>
+          <t>たとえ〜ても</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>…的话就可以</t>
+          <t>即使...也...</t>
         </is>
       </c>
       <c r="D48" t="inlineStr"/>
@@ -1353,15 +1329,19 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>あらかじめ</t>
+          <t>という気</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>预先，事先</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr"/>
+          <t>...样的感觉</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>というき</t>
+        </is>
+      </c>
       <c r="E49" t="inlineStr"/>
     </row>
     <row r="50">
@@ -1370,12 +1350,12 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>どのように</t>
+          <t>しかも</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>怎样地，如何地</t>
+          <t>而且</t>
         </is>
       </c>
       <c r="D50" t="inlineStr"/>
@@ -1383,24 +1363,24 @@
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>〜を〜として</t>
+          <t>活躍</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>把...当作...</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr"/>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>“～を～にする”把…作为</t>
-        </is>
-      </c>
+          <t>活跃，大显身手</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>かつやく</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -1408,38 +1388,34 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>という気</t>
+          <t>のうち</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>...样的感觉</t>
-        </is>
-      </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>というき</t>
-        </is>
-      </c>
+          <t>...之中</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr"/>
       <c r="E52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>気にしない</t>
+          <t>相性が悪い</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>不在意</t>
+          <t>(两人)合不来</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>きにしない</t>
+          <t>あいしょうがわるい</t>
         </is>
       </c>
       <c r="E53" t="inlineStr"/>
@@ -1450,36 +1426,36 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>あふれる</t>
+          <t>通りに</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>溢出，充满</t>
-        </is>
-      </c>
-      <c r="D54" t="inlineStr"/>
+          <t>按照...</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>とおりに</t>
+        </is>
+      </c>
       <c r="E54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>丈夫</t>
+          <t>とよい</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>结实的；健康的</t>
-        </is>
-      </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>じょうぶ</t>
-        </is>
-      </c>
+          <t>…的话就可以</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr"/>
       <c r="E55" t="inlineStr"/>
     </row>
     <row r="56">
@@ -1488,12 +1464,12 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>なおす</t>
+          <t>どこか</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>修理；改正</t>
+          <t>某处，总觉得</t>
         </is>
       </c>
       <c r="D56" t="inlineStr"/>
@@ -1501,37 +1477,33 @@
     </row>
     <row r="57">
       <c r="A57" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>に対し</t>
+          <t>N+による+N</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>对于...</t>
-        </is>
-      </c>
-      <c r="D57" t="inlineStr">
-        <is>
-          <t>にたいし</t>
-        </is>
-      </c>
+          <t>由...（所造成的）...</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr"/>
       <c r="E57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>そうして〜</t>
+          <t>ととらえる</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>这么做…</t>
+          <t>视为...，理解为...</t>
         </is>
       </c>
       <c r="D58" t="inlineStr"/>
@@ -1539,16 +1511,16 @@
     </row>
     <row r="59">
       <c r="A59" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>〜のは〜せいだ</t>
+          <t>どのように</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>之所以…都怪…</t>
+          <t>怎样地，如何地</t>
         </is>
       </c>
       <c r="D59" t="inlineStr"/>
@@ -1560,15 +1532,19 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>せずに</t>
+          <t>納得</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>不做...就...（书面语）</t>
-        </is>
-      </c>
-      <c r="D60" t="inlineStr"/>
+          <t>认同，信服</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>なっとく</t>
+        </is>
+      </c>
       <c r="E60" t="inlineStr"/>
     </row>
     <row r="61">
@@ -1577,19 +1553,15 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>与える</t>
+          <t>〜に気づく</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>给予，赋予</t>
-        </is>
-      </c>
-      <c r="D61" t="inlineStr">
-        <is>
-          <t>あたえる</t>
-        </is>
-      </c>
+          <t>发现…</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr"/>
       <c r="E61" t="inlineStr"/>
     </row>
     <row r="62">
@@ -1598,15 +1570,19 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>なにもかも</t>
+          <t>何とか</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>一切，所有</t>
-        </is>
-      </c>
-      <c r="D62" t="inlineStr"/>
+          <t>设法，总算</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>なんとか</t>
+        </is>
+      </c>
       <c r="E62" t="inlineStr"/>
     </row>
     <row r="63">
@@ -1615,15 +1591,19 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>やってくる</t>
+          <t>出来上がる</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>到来；做过来</t>
-        </is>
-      </c>
-      <c r="D63" t="inlineStr"/>
+          <t>完成，做好</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>できあがる</t>
+        </is>
+      </c>
       <c r="E63" t="inlineStr"/>
     </row>
     <row r="64">
@@ -1632,32 +1612,40 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>たとえ〜ても</t>
+          <t>見本</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>即使...也...</t>
-        </is>
-      </c>
-      <c r="D64" t="inlineStr"/>
+          <t>样本，样品</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>みほん</t>
+        </is>
+      </c>
       <c r="E64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>らしい</t>
+          <t>を生かして</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>好像...；很有...的风格</t>
-        </is>
-      </c>
-      <c r="D65" t="inlineStr"/>
+          <t>发挥...，利用...</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>をいかして</t>
+        </is>
+      </c>
       <c r="E65" t="inlineStr"/>
     </row>
     <row r="66">
@@ -1666,12 +1654,12 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>なんとかなる</t>
+          <t>どんなに</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>总会有办法的</t>
+          <t>无论多么...</t>
         </is>
       </c>
       <c r="D66" t="inlineStr"/>
@@ -1683,15 +1671,19 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>それなのに</t>
+          <t>受け取る</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>尽管如此，可是...</t>
-        </is>
-      </c>
-      <c r="D67" t="inlineStr"/>
+          <t>接收，领取；理解</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>うけとる</t>
+        </is>
+      </c>
       <c r="E67" t="inlineStr"/>
     </row>
     <row r="68">
@@ -1700,87 +1692,99 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>〜ないだろうか</t>
+          <t>たまに</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>是否…</t>
+          <t>偶尔</t>
         </is>
       </c>
       <c r="D68" t="inlineStr"/>
-      <c r="E68" t="inlineStr"/>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>“たまたま”偶然；碰巧</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>〜に気づく</t>
+          <t>新たに</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>发现…</t>
-        </is>
-      </c>
-      <c r="D69" t="inlineStr"/>
+          <t>新，重新</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>あらたに</t>
+        </is>
+      </c>
       <c r="E69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>たまに</t>
+          <t>らしい</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>偶尔</t>
+          <t>好像...；很有...的风格</t>
         </is>
       </c>
       <c r="D70" t="inlineStr"/>
-      <c r="E70" t="inlineStr">
-        <is>
-          <t>“たまたま”偶然；碰巧</t>
-        </is>
-      </c>
+      <c r="E70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>N+による+N</t>
+          <t>身につく</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>由...（所造成的）...</t>
-        </is>
-      </c>
-      <c r="D71" t="inlineStr"/>
+          <t>掌握，学会</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>みにつく</t>
+        </is>
+      </c>
       <c r="E71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>なんらか</t>
+          <t>に対し</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>某些，某种</t>
-        </is>
-      </c>
-      <c r="D72" t="inlineStr"/>
+          <t>对于...</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>にたいし</t>
+        </is>
+      </c>
       <c r="E72" t="inlineStr"/>
     </row>
     <row r="73">
@@ -1789,19 +1793,15 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>簡単に</t>
+          <t>とらえる</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>轻易地</t>
-        </is>
-      </c>
-      <c r="D73" t="inlineStr">
-        <is>
-          <t>かんたんに</t>
-        </is>
-      </c>
+          <t>捕捉，理解</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr"/>
       <c r="E73" t="inlineStr"/>
     </row>
     <row r="74">
@@ -1810,36 +1810,36 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>新たに</t>
+          <t>〜のは〜せいだ</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>新，重新</t>
-        </is>
-      </c>
-      <c r="D74" t="inlineStr">
-        <is>
-          <t>あらたに</t>
-        </is>
-      </c>
+          <t>之所以…都怪…</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr"/>
       <c r="E74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>どこか</t>
+          <t>気にしない</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>某处，总觉得</t>
-        </is>
-      </c>
-      <c r="D75" t="inlineStr"/>
+          <t>不在意</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>きにしない</t>
+        </is>
+      </c>
       <c r="E75" t="inlineStr"/>
     </row>
     <row r="76">
@@ -1848,15 +1848,19 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>はずがない</t>
+          <t>気が合う</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>不可能...</t>
-        </is>
-      </c>
-      <c r="D76" t="inlineStr"/>
+          <t>合得来</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>きがあう</t>
+        </is>
+      </c>
       <c r="E76" t="inlineStr"/>
     </row>
     <row r="77">
@@ -1865,17 +1869,17 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>見つける</t>
+          <t>旅先</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>找到（主观动作）</t>
+          <t>旅途目的地</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>みつける</t>
+          <t>たびさき</t>
         </is>
       </c>
       <c r="E77" t="inlineStr"/>
@@ -1886,33 +1890,33 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>見つかる</t>
+          <t>数量詞+ずつ</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>被找到（客观状态）</t>
+          <t>每...（数量）</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>みつかる</t>
+          <t>すうりょうし+ずつ</t>
         </is>
       </c>
       <c r="E78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>どんなに</t>
+          <t>ぜひ</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>无论多么...</t>
+          <t>一定，务必</t>
         </is>
       </c>
       <c r="D79" t="inlineStr"/>
@@ -1924,17 +1928,17 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>無駄</t>
+          <t>簡単に</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>浪费，徒劳</t>
+          <t>轻易地</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>むだ</t>
+          <t>かんたんに</t>
         </is>
       </c>
       <c r="E80" t="inlineStr"/>
@@ -1945,17 +1949,17 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>旅先</t>
+          <t>見つける</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>旅途目的地</t>
+          <t>找到（主观动作）</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>たびさき</t>
+          <t>みつける</t>
         </is>
       </c>
       <c r="E81" t="inlineStr"/>
@@ -1966,17 +1970,17 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>気が合う</t>
+          <t>見つかる</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>合得来</t>
+          <t>被找到（客观状态）</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>きがあう</t>
+          <t>みつかる</t>
         </is>
       </c>
       <c r="E82" t="inlineStr"/>
@@ -1987,61 +1991,57 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>何が起こる</t>
+          <t>〜に限り</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>发生某事</t>
+          <t>限于...，只有...</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>なにがおこる</t>
+          <t>〜にかぎり</t>
         </is>
       </c>
       <c r="E83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>を生かして</t>
+          <t>無駄</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>发挥...，利用...</t>
+          <t>浪费，徒劳</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>をいかして</t>
+          <t>むだ</t>
         </is>
       </c>
       <c r="E84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>出来上がる</t>
+          <t>によって</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>完成，做好</t>
-        </is>
-      </c>
-      <c r="D85" t="inlineStr">
-        <is>
-          <t>できあがる</t>
-        </is>
-      </c>
+          <t>根据...；由于...</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr"/>
       <c r="E85" t="inlineStr"/>
     </row>
     <row r="86">
@@ -2050,34 +2050,38 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>というのは</t>
+          <t>〜を〜として</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>所谓...；说的是...</t>
+          <t>把...当作...</t>
         </is>
       </c>
       <c r="D86" t="inlineStr"/>
-      <c r="E86" t="inlineStr"/>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>“～を～にする”把…作为</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>何とか</t>
+          <t>積み重ねる</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>设法，总算</t>
+          <t>积累</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>なんとか</t>
+          <t>つみかさねる</t>
         </is>
       </c>
       <c r="E87" t="inlineStr"/>
@@ -2088,15 +2092,19 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>であろう</t>
+          <t>役目</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>...吧（「だろう」的书面语）</t>
-        </is>
-      </c>
-      <c r="D88" t="inlineStr"/>
+          <t>作用，职责</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>やくめ</t>
+        </is>
+      </c>
       <c r="E88" t="inlineStr"/>
     </row>
     <row r="89">
@@ -2105,40 +2113,32 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>任せる</t>
+          <t>はずがない</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>委托，托付</t>
-        </is>
-      </c>
-      <c r="D89" t="inlineStr">
-        <is>
-          <t>まかせる</t>
-        </is>
-      </c>
+          <t>不可能...</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr"/>
       <c r="E89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>着実に</t>
+          <t>および</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>切实地，踏实地</t>
-        </is>
-      </c>
-      <c r="D90" t="inlineStr">
-        <is>
-          <t>ちゃくじつに</t>
-        </is>
-      </c>
+          <t>以及，和</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr"/>
       <c r="E90" t="inlineStr"/>
     </row>
     <row r="91">
@@ -2147,38 +2147,34 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>与える</t>
+          <t>いけない</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>给予...</t>
-        </is>
-      </c>
-      <c r="D91" t="inlineStr">
-        <is>
-          <t>あたえる</t>
-        </is>
-      </c>
+          <t>不行，不可以</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr"/>
       <c r="E91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>通りに</t>
+          <t>与える</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>按照...</t>
+          <t>给予...</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>とおりに</t>
+          <t>あたえる</t>
         </is>
       </c>
       <c r="E92" t="inlineStr"/>
@@ -2189,40 +2185,36 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>繰り返す</t>
+          <t>任せる</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>重复</t>
+          <t>委托，托付</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>くりかえす</t>
+          <t>まかせる</t>
         </is>
       </c>
       <c r="E93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>見本</t>
+          <t>であろう</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>样本，样品</t>
-        </is>
-      </c>
-      <c r="D94" t="inlineStr">
-        <is>
-          <t>みほん</t>
-        </is>
-      </c>
+          <t>...吧（「だろう」的书面语）</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr"/>
       <c r="E94" t="inlineStr"/>
     </row>
     <row r="95">
@@ -2231,36 +2223,36 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>最善</t>
+          <t>というのは</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>最好的，万全的</t>
-        </is>
-      </c>
-      <c r="D95" t="inlineStr">
-        <is>
-          <t>さいぜん</t>
-        </is>
-      </c>
+          <t>所谓...；说的是...</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr"/>
       <c r="E95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>つかむ</t>
+          <t>繰り返す</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>抓住，掌握</t>
-        </is>
-      </c>
-      <c r="D96" t="inlineStr"/>
+          <t>重复</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>くりかえす</t>
+        </is>
+      </c>
       <c r="E96" t="inlineStr"/>
     </row>
     <row r="97">
@@ -2269,17 +2261,17 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>身につく</t>
+          <t>周り</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>掌握，学会</t>
+          <t>周围</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>みにつく</t>
+          <t>まわり</t>
         </is>
       </c>
       <c r="E97" t="inlineStr"/>
@@ -2290,36 +2282,36 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>いけない</t>
+          <t>最善</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>不行，不可以</t>
-        </is>
-      </c>
-      <c r="D98" t="inlineStr"/>
+          <t>最好的，万全的</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>さいぜん</t>
+        </is>
+      </c>
       <c r="E98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>納得</t>
+          <t>なにか</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>认同，信服</t>
-        </is>
-      </c>
-      <c r="D99" t="inlineStr">
-        <is>
-          <t>なっとく</t>
-        </is>
-      </c>
+          <t>什么，某些</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr"/>
       <c r="E99" t="inlineStr"/>
     </row>
     <row r="100">
@@ -2328,17 +2320,17 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>積み重ねる</t>
+          <t>改める</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>积累</t>
+          <t>重新</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>つみかさねる</t>
+          <t>あらためる</t>
         </is>
       </c>
       <c r="E100" t="inlineStr"/>
@@ -2362,16 +2354,16 @@
     </row>
     <row r="102">
       <c r="A102" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>いずれ</t>
+          <t>そのもの</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>反正，早晚</t>
+          <t>本身，自身</t>
         </is>
       </c>
       <c r="D102" t="inlineStr"/>
@@ -2383,12 +2375,12 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>そのもの</t>
+          <t>たとえば</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>本身，自身</t>
+          <t>例如</t>
         </is>
       </c>
       <c r="D103" t="inlineStr"/>
@@ -2400,33 +2392,29 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>役目</t>
+          <t>それぞれ</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>作用，职责</t>
-        </is>
-      </c>
-      <c r="D104" t="inlineStr">
-        <is>
-          <t>やくめ</t>
-        </is>
-      </c>
+          <t>各自，分别</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr"/>
       <c r="E104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>のほかに</t>
+          <t>どちらも…</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>除...之外</t>
+          <t>无论哪一个都…</t>
         </is>
       </c>
       <c r="D105" t="inlineStr"/>
@@ -2438,15 +2426,19 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>〜とする</t>
+          <t>何が起こる</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>假如…</t>
-        </is>
-      </c>
-      <c r="D106" t="inlineStr"/>
+          <t>发生某事</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>なにがおこる</t>
+        </is>
+      </c>
       <c r="E106" t="inlineStr"/>
     </row>
     <row r="107">
@@ -2455,32 +2447,40 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>たとえば</t>
+          <t>身につく</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>例如</t>
-        </is>
-      </c>
-      <c r="D107" t="inlineStr"/>
+          <t>掌握，学会</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>みにつく</t>
+        </is>
+      </c>
       <c r="E107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>Vる+のか</t>
+          <t>丈夫</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>是否…</t>
-        </is>
-      </c>
-      <c r="D108" t="inlineStr"/>
+          <t>结实的；健康的</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>じょうぶ</t>
+        </is>
+      </c>
       <c r="E108" t="inlineStr"/>
     </row>
   </sheetData>

</xml_diff>